<commit_message>
Finalize Coursemark task and DropLine v6.0.3 evidence
</commit_message>
<xml_diff>
--- a/deliverables/dropline-four-lite/final-package/qc/DropLine_Four_Lite_RL_Scorecard.xlsx
+++ b/deliverables/dropline-four-lite/final-package/qc/DropLine_Four_Lite_RL_Scorecard.xlsx
@@ -15,7 +15,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -27,27 +27,96 @@
       <color theme="1"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0019324D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C9D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C9D6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7C9D6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7C9D6"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -323,1154 +392,178 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8.710000000000001" customWidth="1" style="2" min="1" max="26"/>
+    <col width="31" customWidth="1" style="2" min="1" max="1"/>
+    <col width="112" customWidth="1" style="2" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="2">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>DropLine Four Lite — RL Task Quality Scorecard — Result</t>
         </is>
       </c>
+      <c r="B1" s="4" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Headline verdict</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>CONDITIONAL ACCEPT</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Headline verdict</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>CONDITIONAL ACCEPT</t>
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Weighted score (equal weight)</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>50 / 58 = 86.2 %</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Weighted score (equal weight)</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>52 / 58 = 89.7 %</t>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Criteria in template</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>30 criteria present in sheet</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Criteria in template</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>30 criteria present in sheet</t>
-        </is>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Applicable (non-blank)</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Applicable (non-blank)</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>29</v>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>N/A (blank, excluded)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>D5 (1 criterion)</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>N/A (blank, excluded)</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>D5 (1 criterion)</t>
-        </is>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Passes (2)</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Passes (2)</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>23</v>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Partials (1)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>B1, C2, D4, E1, E2, E3, F1, F2 (8 criteria)</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Partials (1)</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>B1, D1, D4, E1, F1, F2 (6 criteria)</t>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Fails (0)</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Fails (0)</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>GATE VERDICT</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>No criterion scores 0; evidence/hash/network/statistical limitations keep the result conditional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Oracle run</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Exact v6.0.3 golden artifact -&gt; reward 1.0000 (22/22 criteria)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>GATE VERDICT</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>No gate at 0 -&gt; NOT rejected; D4 and E1 are Partial -&gt; CONDITIONAL ACCEPT</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Oracle run</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>Final v6.0.3 golden artifact -&gt; reward 1.0000 (22/22 criteria)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>GPT-5.4-mini run</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t>Untouched artifact -&gt; reward 0.3642 (constraints 1.0, functional 0.4737, render 1.0, polish 0.2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Exact v6.0.3 GPT-5.4-mini -&gt; reward 0.5390 (R 1.0, C 1.0, F 0.6316, P 0.4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Claude Haiku 4.5 run</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>Untouched artifact -&gt; hard-gated reward 0.0000; raw functional 0.6842</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Exact v6.0.3 Claude Haiku 4.5 -&gt; reward 0.3327 (R 1.0, C 1.0, F 0.4211, P 0.2); model-caused exit 143</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>No-op run</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Executable no-op -&gt; reward 0.0000 with no_op=1</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="2"/>
-    <row r="22" ht="15.75" customHeight="1" s="2"/>
-    <row r="23" ht="15.75" customHeight="1" s="2"/>
-    <row r="24" ht="15.75" customHeight="1" s="2"/>
-    <row r="25" ht="15.75" customHeight="1" s="2"/>
-    <row r="26" ht="15.75" customHeight="1" s="2"/>
-    <row r="27" ht="15.75" customHeight="1" s="2"/>
-    <row r="28" ht="15.75" customHeight="1" s="2"/>
-    <row r="29" ht="15.75" customHeight="1" s="2"/>
-    <row r="30" ht="15.75" customHeight="1" s="2"/>
-    <row r="31" ht="15.75" customHeight="1" s="2"/>
-    <row r="32" ht="15.75" customHeight="1" s="2"/>
-    <row r="33" ht="15.75" customHeight="1" s="2"/>
-    <row r="34" ht="15.75" customHeight="1" s="2"/>
-    <row r="35" ht="15.75" customHeight="1" s="2"/>
-    <row r="36" ht="15.75" customHeight="1" s="2"/>
-    <row r="37" ht="15.75" customHeight="1" s="2"/>
-    <row r="38" ht="15.75" customHeight="1" s="2"/>
-    <row r="39" ht="15.75" customHeight="1" s="2"/>
-    <row r="40" ht="15.75" customHeight="1" s="2"/>
-    <row r="41" ht="15.75" customHeight="1" s="2"/>
-    <row r="42" ht="15.75" customHeight="1" s="2"/>
-    <row r="43" ht="15.75" customHeight="1" s="2"/>
-    <row r="44" ht="15.75" customHeight="1" s="2"/>
-    <row r="45" ht="15.75" customHeight="1" s="2"/>
-    <row r="46" ht="15.75" customHeight="1" s="2"/>
-    <row r="47" ht="15.75" customHeight="1" s="2"/>
-    <row r="48" ht="15.75" customHeight="1" s="2"/>
-    <row r="49" ht="15.75" customHeight="1" s="2"/>
-    <row r="50" ht="15.75" customHeight="1" s="2"/>
-    <row r="51" ht="15.75" customHeight="1" s="2"/>
-    <row r="52" ht="15.75" customHeight="1" s="2"/>
-    <row r="53" ht="15.75" customHeight="1" s="2"/>
-    <row r="54" ht="15.75" customHeight="1" s="2"/>
-    <row r="55" ht="15.75" customHeight="1" s="2"/>
-    <row r="56" ht="15.75" customHeight="1" s="2"/>
-    <row r="57" ht="15.75" customHeight="1" s="2"/>
-    <row r="58" ht="15.75" customHeight="1" s="2"/>
-    <row r="59" ht="15.75" customHeight="1" s="2"/>
-    <row r="60" ht="15.75" customHeight="1" s="2"/>
-    <row r="61" ht="15.75" customHeight="1" s="2"/>
-    <row r="62" ht="15.75" customHeight="1" s="2"/>
-    <row r="63" ht="15.75" customHeight="1" s="2"/>
-    <row r="64" ht="15.75" customHeight="1" s="2"/>
-    <row r="65" ht="15.75" customHeight="1" s="2"/>
-    <row r="66" ht="15.75" customHeight="1" s="2"/>
-    <row r="67" ht="15.75" customHeight="1" s="2"/>
-    <row r="68" ht="15.75" customHeight="1" s="2"/>
-    <row r="69" ht="15.75" customHeight="1" s="2"/>
-    <row r="70" ht="15.75" customHeight="1" s="2"/>
-    <row r="71" ht="15.75" customHeight="1" s="2"/>
-    <row r="72" ht="15.75" customHeight="1" s="2"/>
-    <row r="73" ht="15.75" customHeight="1" s="2"/>
-    <row r="74" ht="15.75" customHeight="1" s="2"/>
-    <row r="75" ht="15.75" customHeight="1" s="2"/>
-    <row r="76" ht="15.75" customHeight="1" s="2"/>
-    <row r="77" ht="15.75" customHeight="1" s="2"/>
-    <row r="78" ht="15.75" customHeight="1" s="2"/>
-    <row r="79" ht="15.75" customHeight="1" s="2"/>
-    <row r="80" ht="15.75" customHeight="1" s="2"/>
-    <row r="81" ht="15.75" customHeight="1" s="2"/>
-    <row r="82" ht="15.75" customHeight="1" s="2"/>
-    <row r="83" ht="15.75" customHeight="1" s="2"/>
-    <row r="84" ht="15.75" customHeight="1" s="2"/>
-    <row r="85" ht="15.75" customHeight="1" s="2"/>
-    <row r="86" ht="15.75" customHeight="1" s="2"/>
-    <row r="87" ht="15.75" customHeight="1" s="2"/>
-    <row r="88" ht="15.75" customHeight="1" s="2"/>
-    <row r="89" ht="15.75" customHeight="1" s="2"/>
-    <row r="90" ht="15.75" customHeight="1" s="2"/>
-    <row r="91" ht="15.75" customHeight="1" s="2"/>
-    <row r="92" ht="15.75" customHeight="1" s="2"/>
-    <row r="93" ht="15.75" customHeight="1" s="2"/>
-    <row r="94" ht="15.75" customHeight="1" s="2"/>
-    <row r="95" ht="15.75" customHeight="1" s="2"/>
-    <row r="96" ht="15.75" customHeight="1" s="2"/>
-    <row r="97" ht="15.75" customHeight="1" s="2"/>
-    <row r="98" ht="15.75" customHeight="1" s="2"/>
-    <row r="99" ht="15.75" customHeight="1" s="2"/>
-    <row r="100" ht="15.75" customHeight="1" s="2"/>
-    <row r="101" ht="15.75" customHeight="1" s="2"/>
-    <row r="102" ht="15.75" customHeight="1" s="2"/>
-    <row r="103" ht="15.75" customHeight="1" s="2"/>
-    <row r="104" ht="15.75" customHeight="1" s="2"/>
-    <row r="105" ht="15.75" customHeight="1" s="2"/>
-    <row r="106" ht="15.75" customHeight="1" s="2"/>
-    <row r="107" ht="15.75" customHeight="1" s="2"/>
-    <row r="108" ht="15.75" customHeight="1" s="2"/>
-    <row r="109" ht="15.75" customHeight="1" s="2"/>
-    <row r="110" ht="15.75" customHeight="1" s="2"/>
-    <row r="111" ht="15.75" customHeight="1" s="2"/>
-    <row r="112" ht="15.75" customHeight="1" s="2"/>
-    <row r="113" ht="15.75" customHeight="1" s="2"/>
-    <row r="114" ht="15.75" customHeight="1" s="2"/>
-    <row r="115" ht="15.75" customHeight="1" s="2"/>
-    <row r="116" ht="15.75" customHeight="1" s="2"/>
-    <row r="117" ht="15.75" customHeight="1" s="2"/>
-    <row r="118" ht="15.75" customHeight="1" s="2"/>
-    <row r="119" ht="15.75" customHeight="1" s="2"/>
-    <row r="120" ht="15.75" customHeight="1" s="2"/>
-    <row r="121" ht="15.75" customHeight="1" s="2"/>
-    <row r="122" ht="15.75" customHeight="1" s="2"/>
-    <row r="123" ht="15.75" customHeight="1" s="2"/>
-    <row r="124" ht="15.75" customHeight="1" s="2"/>
-    <row r="125" ht="15.75" customHeight="1" s="2"/>
-    <row r="126" ht="15.75" customHeight="1" s="2"/>
-    <row r="127" ht="15.75" customHeight="1" s="2"/>
-    <row r="128" ht="15.75" customHeight="1" s="2"/>
-    <row r="129" ht="15.75" customHeight="1" s="2"/>
-    <row r="130" ht="15.75" customHeight="1" s="2"/>
-    <row r="131" ht="15.75" customHeight="1" s="2"/>
-    <row r="132" ht="15.75" customHeight="1" s="2"/>
-    <row r="133" ht="15.75" customHeight="1" s="2"/>
-    <row r="134" ht="15.75" customHeight="1" s="2"/>
-    <row r="135" ht="15.75" customHeight="1" s="2"/>
-    <row r="136" ht="15.75" customHeight="1" s="2"/>
-    <row r="137" ht="15.75" customHeight="1" s="2"/>
-    <row r="138" ht="15.75" customHeight="1" s="2"/>
-    <row r="139" ht="15.75" customHeight="1" s="2"/>
-    <row r="140" ht="15.75" customHeight="1" s="2"/>
-    <row r="141" ht="15.75" customHeight="1" s="2"/>
-    <row r="142" ht="15.75" customHeight="1" s="2"/>
-    <row r="143" ht="15.75" customHeight="1" s="2"/>
-    <row r="144" ht="15.75" customHeight="1" s="2"/>
-    <row r="145" ht="15.75" customHeight="1" s="2"/>
-    <row r="146" ht="15.75" customHeight="1" s="2"/>
-    <row r="147" ht="15.75" customHeight="1" s="2"/>
-    <row r="148" ht="15.75" customHeight="1" s="2"/>
-    <row r="149" ht="15.75" customHeight="1" s="2"/>
-    <row r="150" ht="15.75" customHeight="1" s="2"/>
-    <row r="151" ht="15.75" customHeight="1" s="2"/>
-    <row r="152" ht="15.75" customHeight="1" s="2"/>
-    <row r="153" ht="15.75" customHeight="1" s="2"/>
-    <row r="154" ht="15.75" customHeight="1" s="2"/>
-    <row r="155" ht="15.75" customHeight="1" s="2"/>
-    <row r="156" ht="15.75" customHeight="1" s="2"/>
-    <row r="157" ht="15.75" customHeight="1" s="2"/>
-    <row r="158" ht="15.75" customHeight="1" s="2"/>
-    <row r="159" ht="15.75" customHeight="1" s="2"/>
-    <row r="160" ht="15.75" customHeight="1" s="2"/>
-    <row r="161" ht="15.75" customHeight="1" s="2"/>
-    <row r="162" ht="15.75" customHeight="1" s="2"/>
-    <row r="163" ht="15.75" customHeight="1" s="2"/>
-    <row r="164" ht="15.75" customHeight="1" s="2"/>
-    <row r="165" ht="15.75" customHeight="1" s="2"/>
-    <row r="166" ht="15.75" customHeight="1" s="2"/>
-    <row r="167" ht="15.75" customHeight="1" s="2"/>
-    <row r="168" ht="15.75" customHeight="1" s="2"/>
-    <row r="169" ht="15.75" customHeight="1" s="2"/>
-    <row r="170" ht="15.75" customHeight="1" s="2"/>
-    <row r="171" ht="15.75" customHeight="1" s="2"/>
-    <row r="172" ht="15.75" customHeight="1" s="2"/>
-    <row r="173" ht="15.75" customHeight="1" s="2"/>
-    <row r="174" ht="15.75" customHeight="1" s="2"/>
-    <row r="175" ht="15.75" customHeight="1" s="2"/>
-    <row r="176" ht="15.75" customHeight="1" s="2"/>
-    <row r="177" ht="15.75" customHeight="1" s="2"/>
-    <row r="178" ht="15.75" customHeight="1" s="2"/>
-    <row r="179" ht="15.75" customHeight="1" s="2"/>
-    <row r="180" ht="15.75" customHeight="1" s="2"/>
-    <row r="181" ht="15.75" customHeight="1" s="2"/>
-    <row r="182" ht="15.75" customHeight="1" s="2"/>
-    <row r="183" ht="15.75" customHeight="1" s="2"/>
-    <row r="184" ht="15.75" customHeight="1" s="2"/>
-    <row r="185" ht="15.75" customHeight="1" s="2"/>
-    <row r="186" ht="15.75" customHeight="1" s="2"/>
-    <row r="187" ht="15.75" customHeight="1" s="2"/>
-    <row r="188" ht="15.75" customHeight="1" s="2"/>
-    <row r="189" ht="15.75" customHeight="1" s="2"/>
-    <row r="190" ht="15.75" customHeight="1" s="2"/>
-    <row r="191" ht="15.75" customHeight="1" s="2"/>
-    <row r="192" ht="15.75" customHeight="1" s="2"/>
-    <row r="193" ht="15.75" customHeight="1" s="2"/>
-    <row r="194" ht="15.75" customHeight="1" s="2"/>
-    <row r="195" ht="15.75" customHeight="1" s="2"/>
-    <row r="196" ht="15.75" customHeight="1" s="2"/>
-    <row r="197" ht="15.75" customHeight="1" s="2"/>
-    <row r="198" ht="15.75" customHeight="1" s="2"/>
-    <row r="199" ht="15.75" customHeight="1" s="2"/>
-    <row r="200" ht="15.75" customHeight="1" s="2"/>
-    <row r="201" ht="15.75" customHeight="1" s="2"/>
-    <row r="202" ht="15.75" customHeight="1" s="2"/>
-    <row r="203" ht="15.75" customHeight="1" s="2"/>
-    <row r="204" ht="15.75" customHeight="1" s="2"/>
-    <row r="205" ht="15.75" customHeight="1" s="2"/>
-    <row r="206" ht="15.75" customHeight="1" s="2"/>
-    <row r="207" ht="15.75" customHeight="1" s="2"/>
-    <row r="208" ht="15.75" customHeight="1" s="2"/>
-    <row r="209" ht="15.75" customHeight="1" s="2"/>
-    <row r="210" ht="15.75" customHeight="1" s="2"/>
-    <row r="211" ht="15.75" customHeight="1" s="2"/>
-    <row r="212" ht="15.75" customHeight="1" s="2"/>
-    <row r="213" ht="15.75" customHeight="1" s="2"/>
-    <row r="214" ht="15.75" customHeight="1" s="2"/>
-    <row r="215" ht="15.75" customHeight="1" s="2"/>
-    <row r="216" ht="15.75" customHeight="1" s="2"/>
-    <row r="217" ht="15.75" customHeight="1" s="2"/>
-    <row r="218" ht="15.75" customHeight="1" s="2"/>
-    <row r="219" ht="15.75" customHeight="1" s="2"/>
-    <row r="220" ht="15.75" customHeight="1" s="2"/>
-    <row r="221" ht="15.75" customHeight="1" s="2"/>
-    <row r="222" ht="15.75" customHeight="1" s="2"/>
-    <row r="223" ht="15.75" customHeight="1" s="2"/>
-    <row r="224" ht="15.75" customHeight="1" s="2"/>
-    <row r="225" ht="15.75" customHeight="1" s="2"/>
-    <row r="226" ht="15.75" customHeight="1" s="2"/>
-    <row r="227" ht="15.75" customHeight="1" s="2"/>
-    <row r="228" ht="15.75" customHeight="1" s="2"/>
-    <row r="229" ht="15.75" customHeight="1" s="2"/>
-    <row r="230" ht="15.75" customHeight="1" s="2"/>
-    <row r="231" ht="15.75" customHeight="1" s="2"/>
-    <row r="232" ht="15.75" customHeight="1" s="2"/>
-    <row r="233" ht="15.75" customHeight="1" s="2"/>
-    <row r="234" ht="15.75" customHeight="1" s="2"/>
-    <row r="235" ht="15.75" customHeight="1" s="2"/>
-    <row r="236" ht="15.75" customHeight="1" s="2"/>
-    <row r="237" ht="15.75" customHeight="1" s="2"/>
-    <row r="238" ht="15.75" customHeight="1" s="2"/>
-    <row r="239" ht="15.75" customHeight="1" s="2"/>
-    <row r="240" ht="15.75" customHeight="1" s="2"/>
-    <row r="241" ht="15.75" customHeight="1" s="2"/>
-    <row r="242" ht="15.75" customHeight="1" s="2"/>
-    <row r="243" ht="15.75" customHeight="1" s="2"/>
-    <row r="244" ht="15.75" customHeight="1" s="2"/>
-    <row r="245" ht="15.75" customHeight="1" s="2"/>
-    <row r="246" ht="15.75" customHeight="1" s="2"/>
-    <row r="247" ht="15.75" customHeight="1" s="2"/>
-    <row r="248" ht="15.75" customHeight="1" s="2"/>
-    <row r="249" ht="15.75" customHeight="1" s="2"/>
-    <row r="250" ht="15.75" customHeight="1" s="2"/>
-    <row r="251" ht="15.75" customHeight="1" s="2"/>
-    <row r="252" ht="15.75" customHeight="1" s="2"/>
-    <row r="253" ht="15.75" customHeight="1" s="2"/>
-    <row r="254" ht="15.75" customHeight="1" s="2"/>
-    <row r="255" ht="15.75" customHeight="1" s="2"/>
-    <row r="256" ht="15.75" customHeight="1" s="2"/>
-    <row r="257" ht="15.75" customHeight="1" s="2"/>
-    <row r="258" ht="15.75" customHeight="1" s="2"/>
-    <row r="259" ht="15.75" customHeight="1" s="2"/>
-    <row r="260" ht="15.75" customHeight="1" s="2"/>
-    <row r="261" ht="15.75" customHeight="1" s="2"/>
-    <row r="262" ht="15.75" customHeight="1" s="2"/>
-    <row r="263" ht="15.75" customHeight="1" s="2"/>
-    <row r="264" ht="15.75" customHeight="1" s="2"/>
-    <row r="265" ht="15.75" customHeight="1" s="2"/>
-    <row r="266" ht="15.75" customHeight="1" s="2"/>
-    <row r="267" ht="15.75" customHeight="1" s="2"/>
-    <row r="268" ht="15.75" customHeight="1" s="2"/>
-    <row r="269" ht="15.75" customHeight="1" s="2"/>
-    <row r="270" ht="15.75" customHeight="1" s="2"/>
-    <row r="271" ht="15.75" customHeight="1" s="2"/>
-    <row r="272" ht="15.75" customHeight="1" s="2"/>
-    <row r="273" ht="15.75" customHeight="1" s="2"/>
-    <row r="274" ht="15.75" customHeight="1" s="2"/>
-    <row r="275" ht="15.75" customHeight="1" s="2"/>
-    <row r="276" ht="15.75" customHeight="1" s="2"/>
-    <row r="277" ht="15.75" customHeight="1" s="2"/>
-    <row r="278" ht="15.75" customHeight="1" s="2"/>
-    <row r="279" ht="15.75" customHeight="1" s="2"/>
-    <row r="280" ht="15.75" customHeight="1" s="2"/>
-    <row r="281" ht="15.75" customHeight="1" s="2"/>
-    <row r="282" ht="15.75" customHeight="1" s="2"/>
-    <row r="283" ht="15.75" customHeight="1" s="2"/>
-    <row r="284" ht="15.75" customHeight="1" s="2"/>
-    <row r="285" ht="15.75" customHeight="1" s="2"/>
-    <row r="286" ht="15.75" customHeight="1" s="2"/>
-    <row r="287" ht="15.75" customHeight="1" s="2"/>
-    <row r="288" ht="15.75" customHeight="1" s="2"/>
-    <row r="289" ht="15.75" customHeight="1" s="2"/>
-    <row r="290" ht="15.75" customHeight="1" s="2"/>
-    <row r="291" ht="15.75" customHeight="1" s="2"/>
-    <row r="292" ht="15.75" customHeight="1" s="2"/>
-    <row r="293" ht="15.75" customHeight="1" s="2"/>
-    <row r="294" ht="15.75" customHeight="1" s="2"/>
-    <row r="295" ht="15.75" customHeight="1" s="2"/>
-    <row r="296" ht="15.75" customHeight="1" s="2"/>
-    <row r="297" ht="15.75" customHeight="1" s="2"/>
-    <row r="298" ht="15.75" customHeight="1" s="2"/>
-    <row r="299" ht="15.75" customHeight="1" s="2"/>
-    <row r="300" ht="15.75" customHeight="1" s="2"/>
-    <row r="301" ht="15.75" customHeight="1" s="2"/>
-    <row r="302" ht="15.75" customHeight="1" s="2"/>
-    <row r="303" ht="15.75" customHeight="1" s="2"/>
-    <row r="304" ht="15.75" customHeight="1" s="2"/>
-    <row r="305" ht="15.75" customHeight="1" s="2"/>
-    <row r="306" ht="15.75" customHeight="1" s="2"/>
-    <row r="307" ht="15.75" customHeight="1" s="2"/>
-    <row r="308" ht="15.75" customHeight="1" s="2"/>
-    <row r="309" ht="15.75" customHeight="1" s="2"/>
-    <row r="310" ht="15.75" customHeight="1" s="2"/>
-    <row r="311" ht="15.75" customHeight="1" s="2"/>
-    <row r="312" ht="15.75" customHeight="1" s="2"/>
-    <row r="313" ht="15.75" customHeight="1" s="2"/>
-    <row r="314" ht="15.75" customHeight="1" s="2"/>
-    <row r="315" ht="15.75" customHeight="1" s="2"/>
-    <row r="316" ht="15.75" customHeight="1" s="2"/>
-    <row r="317" ht="15.75" customHeight="1" s="2"/>
-    <row r="318" ht="15.75" customHeight="1" s="2"/>
-    <row r="319" ht="15.75" customHeight="1" s="2"/>
-    <row r="320" ht="15.75" customHeight="1" s="2"/>
-    <row r="321" ht="15.75" customHeight="1" s="2"/>
-    <row r="322" ht="15.75" customHeight="1" s="2"/>
-    <row r="323" ht="15.75" customHeight="1" s="2"/>
-    <row r="324" ht="15.75" customHeight="1" s="2"/>
-    <row r="325" ht="15.75" customHeight="1" s="2"/>
-    <row r="326" ht="15.75" customHeight="1" s="2"/>
-    <row r="327" ht="15.75" customHeight="1" s="2"/>
-    <row r="328" ht="15.75" customHeight="1" s="2"/>
-    <row r="329" ht="15.75" customHeight="1" s="2"/>
-    <row r="330" ht="15.75" customHeight="1" s="2"/>
-    <row r="331" ht="15.75" customHeight="1" s="2"/>
-    <row r="332" ht="15.75" customHeight="1" s="2"/>
-    <row r="333" ht="15.75" customHeight="1" s="2"/>
-    <row r="334" ht="15.75" customHeight="1" s="2"/>
-    <row r="335" ht="15.75" customHeight="1" s="2"/>
-    <row r="336" ht="15.75" customHeight="1" s="2"/>
-    <row r="337" ht="15.75" customHeight="1" s="2"/>
-    <row r="338" ht="15.75" customHeight="1" s="2"/>
-    <row r="339" ht="15.75" customHeight="1" s="2"/>
-    <row r="340" ht="15.75" customHeight="1" s="2"/>
-    <row r="341" ht="15.75" customHeight="1" s="2"/>
-    <row r="342" ht="15.75" customHeight="1" s="2"/>
-    <row r="343" ht="15.75" customHeight="1" s="2"/>
-    <row r="344" ht="15.75" customHeight="1" s="2"/>
-    <row r="345" ht="15.75" customHeight="1" s="2"/>
-    <row r="346" ht="15.75" customHeight="1" s="2"/>
-    <row r="347" ht="15.75" customHeight="1" s="2"/>
-    <row r="348" ht="15.75" customHeight="1" s="2"/>
-    <row r="349" ht="15.75" customHeight="1" s="2"/>
-    <row r="350" ht="15.75" customHeight="1" s="2"/>
-    <row r="351" ht="15.75" customHeight="1" s="2"/>
-    <row r="352" ht="15.75" customHeight="1" s="2"/>
-    <row r="353" ht="15.75" customHeight="1" s="2"/>
-    <row r="354" ht="15.75" customHeight="1" s="2"/>
-    <row r="355" ht="15.75" customHeight="1" s="2"/>
-    <row r="356" ht="15.75" customHeight="1" s="2"/>
-    <row r="357" ht="15.75" customHeight="1" s="2"/>
-    <row r="358" ht="15.75" customHeight="1" s="2"/>
-    <row r="359" ht="15.75" customHeight="1" s="2"/>
-    <row r="360" ht="15.75" customHeight="1" s="2"/>
-    <row r="361" ht="15.75" customHeight="1" s="2"/>
-    <row r="362" ht="15.75" customHeight="1" s="2"/>
-    <row r="363" ht="15.75" customHeight="1" s="2"/>
-    <row r="364" ht="15.75" customHeight="1" s="2"/>
-    <row r="365" ht="15.75" customHeight="1" s="2"/>
-    <row r="366" ht="15.75" customHeight="1" s="2"/>
-    <row r="367" ht="15.75" customHeight="1" s="2"/>
-    <row r="368" ht="15.75" customHeight="1" s="2"/>
-    <row r="369" ht="15.75" customHeight="1" s="2"/>
-    <row r="370" ht="15.75" customHeight="1" s="2"/>
-    <row r="371" ht="15.75" customHeight="1" s="2"/>
-    <row r="372" ht="15.75" customHeight="1" s="2"/>
-    <row r="373" ht="15.75" customHeight="1" s="2"/>
-    <row r="374" ht="15.75" customHeight="1" s="2"/>
-    <row r="375" ht="15.75" customHeight="1" s="2"/>
-    <row r="376" ht="15.75" customHeight="1" s="2"/>
-    <row r="377" ht="15.75" customHeight="1" s="2"/>
-    <row r="378" ht="15.75" customHeight="1" s="2"/>
-    <row r="379" ht="15.75" customHeight="1" s="2"/>
-    <row r="380" ht="15.75" customHeight="1" s="2"/>
-    <row r="381" ht="15.75" customHeight="1" s="2"/>
-    <row r="382" ht="15.75" customHeight="1" s="2"/>
-    <row r="383" ht="15.75" customHeight="1" s="2"/>
-    <row r="384" ht="15.75" customHeight="1" s="2"/>
-    <row r="385" ht="15.75" customHeight="1" s="2"/>
-    <row r="386" ht="15.75" customHeight="1" s="2"/>
-    <row r="387" ht="15.75" customHeight="1" s="2"/>
-    <row r="388" ht="15.75" customHeight="1" s="2"/>
-    <row r="389" ht="15.75" customHeight="1" s="2"/>
-    <row r="390" ht="15.75" customHeight="1" s="2"/>
-    <row r="391" ht="15.75" customHeight="1" s="2"/>
-    <row r="392" ht="15.75" customHeight="1" s="2"/>
-    <row r="393" ht="15.75" customHeight="1" s="2"/>
-    <row r="394" ht="15.75" customHeight="1" s="2"/>
-    <row r="395" ht="15.75" customHeight="1" s="2"/>
-    <row r="396" ht="15.75" customHeight="1" s="2"/>
-    <row r="397" ht="15.75" customHeight="1" s="2"/>
-    <row r="398" ht="15.75" customHeight="1" s="2"/>
-    <row r="399" ht="15.75" customHeight="1" s="2"/>
-    <row r="400" ht="15.75" customHeight="1" s="2"/>
-    <row r="401" ht="15.75" customHeight="1" s="2"/>
-    <row r="402" ht="15.75" customHeight="1" s="2"/>
-    <row r="403" ht="15.75" customHeight="1" s="2"/>
-    <row r="404" ht="15.75" customHeight="1" s="2"/>
-    <row r="405" ht="15.75" customHeight="1" s="2"/>
-    <row r="406" ht="15.75" customHeight="1" s="2"/>
-    <row r="407" ht="15.75" customHeight="1" s="2"/>
-    <row r="408" ht="15.75" customHeight="1" s="2"/>
-    <row r="409" ht="15.75" customHeight="1" s="2"/>
-    <row r="410" ht="15.75" customHeight="1" s="2"/>
-    <row r="411" ht="15.75" customHeight="1" s="2"/>
-    <row r="412" ht="15.75" customHeight="1" s="2"/>
-    <row r="413" ht="15.75" customHeight="1" s="2"/>
-    <row r="414" ht="15.75" customHeight="1" s="2"/>
-    <row r="415" ht="15.75" customHeight="1" s="2"/>
-    <row r="416" ht="15.75" customHeight="1" s="2"/>
-    <row r="417" ht="15.75" customHeight="1" s="2"/>
-    <row r="418" ht="15.75" customHeight="1" s="2"/>
-    <row r="419" ht="15.75" customHeight="1" s="2"/>
-    <row r="420" ht="15.75" customHeight="1" s="2"/>
-    <row r="421" ht="15.75" customHeight="1" s="2"/>
-    <row r="422" ht="15.75" customHeight="1" s="2"/>
-    <row r="423" ht="15.75" customHeight="1" s="2"/>
-    <row r="424" ht="15.75" customHeight="1" s="2"/>
-    <row r="425" ht="15.75" customHeight="1" s="2"/>
-    <row r="426" ht="15.75" customHeight="1" s="2"/>
-    <row r="427" ht="15.75" customHeight="1" s="2"/>
-    <row r="428" ht="15.75" customHeight="1" s="2"/>
-    <row r="429" ht="15.75" customHeight="1" s="2"/>
-    <row r="430" ht="15.75" customHeight="1" s="2"/>
-    <row r="431" ht="15.75" customHeight="1" s="2"/>
-    <row r="432" ht="15.75" customHeight="1" s="2"/>
-    <row r="433" ht="15.75" customHeight="1" s="2"/>
-    <row r="434" ht="15.75" customHeight="1" s="2"/>
-    <row r="435" ht="15.75" customHeight="1" s="2"/>
-    <row r="436" ht="15.75" customHeight="1" s="2"/>
-    <row r="437" ht="15.75" customHeight="1" s="2"/>
-    <row r="438" ht="15.75" customHeight="1" s="2"/>
-    <row r="439" ht="15.75" customHeight="1" s="2"/>
-    <row r="440" ht="15.75" customHeight="1" s="2"/>
-    <row r="441" ht="15.75" customHeight="1" s="2"/>
-    <row r="442" ht="15.75" customHeight="1" s="2"/>
-    <row r="443" ht="15.75" customHeight="1" s="2"/>
-    <row r="444" ht="15.75" customHeight="1" s="2"/>
-    <row r="445" ht="15.75" customHeight="1" s="2"/>
-    <row r="446" ht="15.75" customHeight="1" s="2"/>
-    <row r="447" ht="15.75" customHeight="1" s="2"/>
-    <row r="448" ht="15.75" customHeight="1" s="2"/>
-    <row r="449" ht="15.75" customHeight="1" s="2"/>
-    <row r="450" ht="15.75" customHeight="1" s="2"/>
-    <row r="451" ht="15.75" customHeight="1" s="2"/>
-    <row r="452" ht="15.75" customHeight="1" s="2"/>
-    <row r="453" ht="15.75" customHeight="1" s="2"/>
-    <row r="454" ht="15.75" customHeight="1" s="2"/>
-    <row r="455" ht="15.75" customHeight="1" s="2"/>
-    <row r="456" ht="15.75" customHeight="1" s="2"/>
-    <row r="457" ht="15.75" customHeight="1" s="2"/>
-    <row r="458" ht="15.75" customHeight="1" s="2"/>
-    <row r="459" ht="15.75" customHeight="1" s="2"/>
-    <row r="460" ht="15.75" customHeight="1" s="2"/>
-    <row r="461" ht="15.75" customHeight="1" s="2"/>
-    <row r="462" ht="15.75" customHeight="1" s="2"/>
-    <row r="463" ht="15.75" customHeight="1" s="2"/>
-    <row r="464" ht="15.75" customHeight="1" s="2"/>
-    <row r="465" ht="15.75" customHeight="1" s="2"/>
-    <row r="466" ht="15.75" customHeight="1" s="2"/>
-    <row r="467" ht="15.75" customHeight="1" s="2"/>
-    <row r="468" ht="15.75" customHeight="1" s="2"/>
-    <row r="469" ht="15.75" customHeight="1" s="2"/>
-    <row r="470" ht="15.75" customHeight="1" s="2"/>
-    <row r="471" ht="15.75" customHeight="1" s="2"/>
-    <row r="472" ht="15.75" customHeight="1" s="2"/>
-    <row r="473" ht="15.75" customHeight="1" s="2"/>
-    <row r="474" ht="15.75" customHeight="1" s="2"/>
-    <row r="475" ht="15.75" customHeight="1" s="2"/>
-    <row r="476" ht="15.75" customHeight="1" s="2"/>
-    <row r="477" ht="15.75" customHeight="1" s="2"/>
-    <row r="478" ht="15.75" customHeight="1" s="2"/>
-    <row r="479" ht="15.75" customHeight="1" s="2"/>
-    <row r="480" ht="15.75" customHeight="1" s="2"/>
-    <row r="481" ht="15.75" customHeight="1" s="2"/>
-    <row r="482" ht="15.75" customHeight="1" s="2"/>
-    <row r="483" ht="15.75" customHeight="1" s="2"/>
-    <row r="484" ht="15.75" customHeight="1" s="2"/>
-    <row r="485" ht="15.75" customHeight="1" s="2"/>
-    <row r="486" ht="15.75" customHeight="1" s="2"/>
-    <row r="487" ht="15.75" customHeight="1" s="2"/>
-    <row r="488" ht="15.75" customHeight="1" s="2"/>
-    <row r="489" ht="15.75" customHeight="1" s="2"/>
-    <row r="490" ht="15.75" customHeight="1" s="2"/>
-    <row r="491" ht="15.75" customHeight="1" s="2"/>
-    <row r="492" ht="15.75" customHeight="1" s="2"/>
-    <row r="493" ht="15.75" customHeight="1" s="2"/>
-    <row r="494" ht="15.75" customHeight="1" s="2"/>
-    <row r="495" ht="15.75" customHeight="1" s="2"/>
-    <row r="496" ht="15.75" customHeight="1" s="2"/>
-    <row r="497" ht="15.75" customHeight="1" s="2"/>
-    <row r="498" ht="15.75" customHeight="1" s="2"/>
-    <row r="499" ht="15.75" customHeight="1" s="2"/>
-    <row r="500" ht="15.75" customHeight="1" s="2"/>
-    <row r="501" ht="15.75" customHeight="1" s="2"/>
-    <row r="502" ht="15.75" customHeight="1" s="2"/>
-    <row r="503" ht="15.75" customHeight="1" s="2"/>
-    <row r="504" ht="15.75" customHeight="1" s="2"/>
-    <row r="505" ht="15.75" customHeight="1" s="2"/>
-    <row r="506" ht="15.75" customHeight="1" s="2"/>
-    <row r="507" ht="15.75" customHeight="1" s="2"/>
-    <row r="508" ht="15.75" customHeight="1" s="2"/>
-    <row r="509" ht="15.75" customHeight="1" s="2"/>
-    <row r="510" ht="15.75" customHeight="1" s="2"/>
-    <row r="511" ht="15.75" customHeight="1" s="2"/>
-    <row r="512" ht="15.75" customHeight="1" s="2"/>
-    <row r="513" ht="15.75" customHeight="1" s="2"/>
-    <row r="514" ht="15.75" customHeight="1" s="2"/>
-    <row r="515" ht="15.75" customHeight="1" s="2"/>
-    <row r="516" ht="15.75" customHeight="1" s="2"/>
-    <row r="517" ht="15.75" customHeight="1" s="2"/>
-    <row r="518" ht="15.75" customHeight="1" s="2"/>
-    <row r="519" ht="15.75" customHeight="1" s="2"/>
-    <row r="520" ht="15.75" customHeight="1" s="2"/>
-    <row r="521" ht="15.75" customHeight="1" s="2"/>
-    <row r="522" ht="15.75" customHeight="1" s="2"/>
-    <row r="523" ht="15.75" customHeight="1" s="2"/>
-    <row r="524" ht="15.75" customHeight="1" s="2"/>
-    <row r="525" ht="15.75" customHeight="1" s="2"/>
-    <row r="526" ht="15.75" customHeight="1" s="2"/>
-    <row r="527" ht="15.75" customHeight="1" s="2"/>
-    <row r="528" ht="15.75" customHeight="1" s="2"/>
-    <row r="529" ht="15.75" customHeight="1" s="2"/>
-    <row r="530" ht="15.75" customHeight="1" s="2"/>
-    <row r="531" ht="15.75" customHeight="1" s="2"/>
-    <row r="532" ht="15.75" customHeight="1" s="2"/>
-    <row r="533" ht="15.75" customHeight="1" s="2"/>
-    <row r="534" ht="15.75" customHeight="1" s="2"/>
-    <row r="535" ht="15.75" customHeight="1" s="2"/>
-    <row r="536" ht="15.75" customHeight="1" s="2"/>
-    <row r="537" ht="15.75" customHeight="1" s="2"/>
-    <row r="538" ht="15.75" customHeight="1" s="2"/>
-    <row r="539" ht="15.75" customHeight="1" s="2"/>
-    <row r="540" ht="15.75" customHeight="1" s="2"/>
-    <row r="541" ht="15.75" customHeight="1" s="2"/>
-    <row r="542" ht="15.75" customHeight="1" s="2"/>
-    <row r="543" ht="15.75" customHeight="1" s="2"/>
-    <row r="544" ht="15.75" customHeight="1" s="2"/>
-    <row r="545" ht="15.75" customHeight="1" s="2"/>
-    <row r="546" ht="15.75" customHeight="1" s="2"/>
-    <row r="547" ht="15.75" customHeight="1" s="2"/>
-    <row r="548" ht="15.75" customHeight="1" s="2"/>
-    <row r="549" ht="15.75" customHeight="1" s="2"/>
-    <row r="550" ht="15.75" customHeight="1" s="2"/>
-    <row r="551" ht="15.75" customHeight="1" s="2"/>
-    <row r="552" ht="15.75" customHeight="1" s="2"/>
-    <row r="553" ht="15.75" customHeight="1" s="2"/>
-    <row r="554" ht="15.75" customHeight="1" s="2"/>
-    <row r="555" ht="15.75" customHeight="1" s="2"/>
-    <row r="556" ht="15.75" customHeight="1" s="2"/>
-    <row r="557" ht="15.75" customHeight="1" s="2"/>
-    <row r="558" ht="15.75" customHeight="1" s="2"/>
-    <row r="559" ht="15.75" customHeight="1" s="2"/>
-    <row r="560" ht="15.75" customHeight="1" s="2"/>
-    <row r="561" ht="15.75" customHeight="1" s="2"/>
-    <row r="562" ht="15.75" customHeight="1" s="2"/>
-    <row r="563" ht="15.75" customHeight="1" s="2"/>
-    <row r="564" ht="15.75" customHeight="1" s="2"/>
-    <row r="565" ht="15.75" customHeight="1" s="2"/>
-    <row r="566" ht="15.75" customHeight="1" s="2"/>
-    <row r="567" ht="15.75" customHeight="1" s="2"/>
-    <row r="568" ht="15.75" customHeight="1" s="2"/>
-    <row r="569" ht="15.75" customHeight="1" s="2"/>
-    <row r="570" ht="15.75" customHeight="1" s="2"/>
-    <row r="571" ht="15.75" customHeight="1" s="2"/>
-    <row r="572" ht="15.75" customHeight="1" s="2"/>
-    <row r="573" ht="15.75" customHeight="1" s="2"/>
-    <row r="574" ht="15.75" customHeight="1" s="2"/>
-    <row r="575" ht="15.75" customHeight="1" s="2"/>
-    <row r="576" ht="15.75" customHeight="1" s="2"/>
-    <row r="577" ht="15.75" customHeight="1" s="2"/>
-    <row r="578" ht="15.75" customHeight="1" s="2"/>
-    <row r="579" ht="15.75" customHeight="1" s="2"/>
-    <row r="580" ht="15.75" customHeight="1" s="2"/>
-    <row r="581" ht="15.75" customHeight="1" s="2"/>
-    <row r="582" ht="15.75" customHeight="1" s="2"/>
-    <row r="583" ht="15.75" customHeight="1" s="2"/>
-    <row r="584" ht="15.75" customHeight="1" s="2"/>
-    <row r="585" ht="15.75" customHeight="1" s="2"/>
-    <row r="586" ht="15.75" customHeight="1" s="2"/>
-    <row r="587" ht="15.75" customHeight="1" s="2"/>
-    <row r="588" ht="15.75" customHeight="1" s="2"/>
-    <row r="589" ht="15.75" customHeight="1" s="2"/>
-    <row r="590" ht="15.75" customHeight="1" s="2"/>
-    <row r="591" ht="15.75" customHeight="1" s="2"/>
-    <row r="592" ht="15.75" customHeight="1" s="2"/>
-    <row r="593" ht="15.75" customHeight="1" s="2"/>
-    <row r="594" ht="15.75" customHeight="1" s="2"/>
-    <row r="595" ht="15.75" customHeight="1" s="2"/>
-    <row r="596" ht="15.75" customHeight="1" s="2"/>
-    <row r="597" ht="15.75" customHeight="1" s="2"/>
-    <row r="598" ht="15.75" customHeight="1" s="2"/>
-    <row r="599" ht="15.75" customHeight="1" s="2"/>
-    <row r="600" ht="15.75" customHeight="1" s="2"/>
-    <row r="601" ht="15.75" customHeight="1" s="2"/>
-    <row r="602" ht="15.75" customHeight="1" s="2"/>
-    <row r="603" ht="15.75" customHeight="1" s="2"/>
-    <row r="604" ht="15.75" customHeight="1" s="2"/>
-    <row r="605" ht="15.75" customHeight="1" s="2"/>
-    <row r="606" ht="15.75" customHeight="1" s="2"/>
-    <row r="607" ht="15.75" customHeight="1" s="2"/>
-    <row r="608" ht="15.75" customHeight="1" s="2"/>
-    <row r="609" ht="15.75" customHeight="1" s="2"/>
-    <row r="610" ht="15.75" customHeight="1" s="2"/>
-    <row r="611" ht="15.75" customHeight="1" s="2"/>
-    <row r="612" ht="15.75" customHeight="1" s="2"/>
-    <row r="613" ht="15.75" customHeight="1" s="2"/>
-    <row r="614" ht="15.75" customHeight="1" s="2"/>
-    <row r="615" ht="15.75" customHeight="1" s="2"/>
-    <row r="616" ht="15.75" customHeight="1" s="2"/>
-    <row r="617" ht="15.75" customHeight="1" s="2"/>
-    <row r="618" ht="15.75" customHeight="1" s="2"/>
-    <row r="619" ht="15.75" customHeight="1" s="2"/>
-    <row r="620" ht="15.75" customHeight="1" s="2"/>
-    <row r="621" ht="15.75" customHeight="1" s="2"/>
-    <row r="622" ht="15.75" customHeight="1" s="2"/>
-    <row r="623" ht="15.75" customHeight="1" s="2"/>
-    <row r="624" ht="15.75" customHeight="1" s="2"/>
-    <row r="625" ht="15.75" customHeight="1" s="2"/>
-    <row r="626" ht="15.75" customHeight="1" s="2"/>
-    <row r="627" ht="15.75" customHeight="1" s="2"/>
-    <row r="628" ht="15.75" customHeight="1" s="2"/>
-    <row r="629" ht="15.75" customHeight="1" s="2"/>
-    <row r="630" ht="15.75" customHeight="1" s="2"/>
-    <row r="631" ht="15.75" customHeight="1" s="2"/>
-    <row r="632" ht="15.75" customHeight="1" s="2"/>
-    <row r="633" ht="15.75" customHeight="1" s="2"/>
-    <row r="634" ht="15.75" customHeight="1" s="2"/>
-    <row r="635" ht="15.75" customHeight="1" s="2"/>
-    <row r="636" ht="15.75" customHeight="1" s="2"/>
-    <row r="637" ht="15.75" customHeight="1" s="2"/>
-    <row r="638" ht="15.75" customHeight="1" s="2"/>
-    <row r="639" ht="15.75" customHeight="1" s="2"/>
-    <row r="640" ht="15.75" customHeight="1" s="2"/>
-    <row r="641" ht="15.75" customHeight="1" s="2"/>
-    <row r="642" ht="15.75" customHeight="1" s="2"/>
-    <row r="643" ht="15.75" customHeight="1" s="2"/>
-    <row r="644" ht="15.75" customHeight="1" s="2"/>
-    <row r="645" ht="15.75" customHeight="1" s="2"/>
-    <row r="646" ht="15.75" customHeight="1" s="2"/>
-    <row r="647" ht="15.75" customHeight="1" s="2"/>
-    <row r="648" ht="15.75" customHeight="1" s="2"/>
-    <row r="649" ht="15.75" customHeight="1" s="2"/>
-    <row r="650" ht="15.75" customHeight="1" s="2"/>
-    <row r="651" ht="15.75" customHeight="1" s="2"/>
-    <row r="652" ht="15.75" customHeight="1" s="2"/>
-    <row r="653" ht="15.75" customHeight="1" s="2"/>
-    <row r="654" ht="15.75" customHeight="1" s="2"/>
-    <row r="655" ht="15.75" customHeight="1" s="2"/>
-    <row r="656" ht="15.75" customHeight="1" s="2"/>
-    <row r="657" ht="15.75" customHeight="1" s="2"/>
-    <row r="658" ht="15.75" customHeight="1" s="2"/>
-    <row r="659" ht="15.75" customHeight="1" s="2"/>
-    <row r="660" ht="15.75" customHeight="1" s="2"/>
-    <row r="661" ht="15.75" customHeight="1" s="2"/>
-    <row r="662" ht="15.75" customHeight="1" s="2"/>
-    <row r="663" ht="15.75" customHeight="1" s="2"/>
-    <row r="664" ht="15.75" customHeight="1" s="2"/>
-    <row r="665" ht="15.75" customHeight="1" s="2"/>
-    <row r="666" ht="15.75" customHeight="1" s="2"/>
-    <row r="667" ht="15.75" customHeight="1" s="2"/>
-    <row r="668" ht="15.75" customHeight="1" s="2"/>
-    <row r="669" ht="15.75" customHeight="1" s="2"/>
-    <row r="670" ht="15.75" customHeight="1" s="2"/>
-    <row r="671" ht="15.75" customHeight="1" s="2"/>
-    <row r="672" ht="15.75" customHeight="1" s="2"/>
-    <row r="673" ht="15.75" customHeight="1" s="2"/>
-    <row r="674" ht="15.75" customHeight="1" s="2"/>
-    <row r="675" ht="15.75" customHeight="1" s="2"/>
-    <row r="676" ht="15.75" customHeight="1" s="2"/>
-    <row r="677" ht="15.75" customHeight="1" s="2"/>
-    <row r="678" ht="15.75" customHeight="1" s="2"/>
-    <row r="679" ht="15.75" customHeight="1" s="2"/>
-    <row r="680" ht="15.75" customHeight="1" s="2"/>
-    <row r="681" ht="15.75" customHeight="1" s="2"/>
-    <row r="682" ht="15.75" customHeight="1" s="2"/>
-    <row r="683" ht="15.75" customHeight="1" s="2"/>
-    <row r="684" ht="15.75" customHeight="1" s="2"/>
-    <row r="685" ht="15.75" customHeight="1" s="2"/>
-    <row r="686" ht="15.75" customHeight="1" s="2"/>
-    <row r="687" ht="15.75" customHeight="1" s="2"/>
-    <row r="688" ht="15.75" customHeight="1" s="2"/>
-    <row r="689" ht="15.75" customHeight="1" s="2"/>
-    <row r="690" ht="15.75" customHeight="1" s="2"/>
-    <row r="691" ht="15.75" customHeight="1" s="2"/>
-    <row r="692" ht="15.75" customHeight="1" s="2"/>
-    <row r="693" ht="15.75" customHeight="1" s="2"/>
-    <row r="694" ht="15.75" customHeight="1" s="2"/>
-    <row r="695" ht="15.75" customHeight="1" s="2"/>
-    <row r="696" ht="15.75" customHeight="1" s="2"/>
-    <row r="697" ht="15.75" customHeight="1" s="2"/>
-    <row r="698" ht="15.75" customHeight="1" s="2"/>
-    <row r="699" ht="15.75" customHeight="1" s="2"/>
-    <row r="700" ht="15.75" customHeight="1" s="2"/>
-    <row r="701" ht="15.75" customHeight="1" s="2"/>
-    <row r="702" ht="15.75" customHeight="1" s="2"/>
-    <row r="703" ht="15.75" customHeight="1" s="2"/>
-    <row r="704" ht="15.75" customHeight="1" s="2"/>
-    <row r="705" ht="15.75" customHeight="1" s="2"/>
-    <row r="706" ht="15.75" customHeight="1" s="2"/>
-    <row r="707" ht="15.75" customHeight="1" s="2"/>
-    <row r="708" ht="15.75" customHeight="1" s="2"/>
-    <row r="709" ht="15.75" customHeight="1" s="2"/>
-    <row r="710" ht="15.75" customHeight="1" s="2"/>
-    <row r="711" ht="15.75" customHeight="1" s="2"/>
-    <row r="712" ht="15.75" customHeight="1" s="2"/>
-    <row r="713" ht="15.75" customHeight="1" s="2"/>
-    <row r="714" ht="15.75" customHeight="1" s="2"/>
-    <row r="715" ht="15.75" customHeight="1" s="2"/>
-    <row r="716" ht="15.75" customHeight="1" s="2"/>
-    <row r="717" ht="15.75" customHeight="1" s="2"/>
-    <row r="718" ht="15.75" customHeight="1" s="2"/>
-    <row r="719" ht="15.75" customHeight="1" s="2"/>
-    <row r="720" ht="15.75" customHeight="1" s="2"/>
-    <row r="721" ht="15.75" customHeight="1" s="2"/>
-    <row r="722" ht="15.75" customHeight="1" s="2"/>
-    <row r="723" ht="15.75" customHeight="1" s="2"/>
-    <row r="724" ht="15.75" customHeight="1" s="2"/>
-    <row r="725" ht="15.75" customHeight="1" s="2"/>
-    <row r="726" ht="15.75" customHeight="1" s="2"/>
-    <row r="727" ht="15.75" customHeight="1" s="2"/>
-    <row r="728" ht="15.75" customHeight="1" s="2"/>
-    <row r="729" ht="15.75" customHeight="1" s="2"/>
-    <row r="730" ht="15.75" customHeight="1" s="2"/>
-    <row r="731" ht="15.75" customHeight="1" s="2"/>
-    <row r="732" ht="15.75" customHeight="1" s="2"/>
-    <row r="733" ht="15.75" customHeight="1" s="2"/>
-    <row r="734" ht="15.75" customHeight="1" s="2"/>
-    <row r="735" ht="15.75" customHeight="1" s="2"/>
-    <row r="736" ht="15.75" customHeight="1" s="2"/>
-    <row r="737" ht="15.75" customHeight="1" s="2"/>
-    <row r="738" ht="15.75" customHeight="1" s="2"/>
-    <row r="739" ht="15.75" customHeight="1" s="2"/>
-    <row r="740" ht="15.75" customHeight="1" s="2"/>
-    <row r="741" ht="15.75" customHeight="1" s="2"/>
-    <row r="742" ht="15.75" customHeight="1" s="2"/>
-    <row r="743" ht="15.75" customHeight="1" s="2"/>
-    <row r="744" ht="15.75" customHeight="1" s="2"/>
-    <row r="745" ht="15.75" customHeight="1" s="2"/>
-    <row r="746" ht="15.75" customHeight="1" s="2"/>
-    <row r="747" ht="15.75" customHeight="1" s="2"/>
-    <row r="748" ht="15.75" customHeight="1" s="2"/>
-    <row r="749" ht="15.75" customHeight="1" s="2"/>
-    <row r="750" ht="15.75" customHeight="1" s="2"/>
-    <row r="751" ht="15.75" customHeight="1" s="2"/>
-    <row r="752" ht="15.75" customHeight="1" s="2"/>
-    <row r="753" ht="15.75" customHeight="1" s="2"/>
-    <row r="754" ht="15.75" customHeight="1" s="2"/>
-    <row r="755" ht="15.75" customHeight="1" s="2"/>
-    <row r="756" ht="15.75" customHeight="1" s="2"/>
-    <row r="757" ht="15.75" customHeight="1" s="2"/>
-    <row r="758" ht="15.75" customHeight="1" s="2"/>
-    <row r="759" ht="15.75" customHeight="1" s="2"/>
-    <row r="760" ht="15.75" customHeight="1" s="2"/>
-    <row r="761" ht="15.75" customHeight="1" s="2"/>
-    <row r="762" ht="15.75" customHeight="1" s="2"/>
-    <row r="763" ht="15.75" customHeight="1" s="2"/>
-    <row r="764" ht="15.75" customHeight="1" s="2"/>
-    <row r="765" ht="15.75" customHeight="1" s="2"/>
-    <row r="766" ht="15.75" customHeight="1" s="2"/>
-    <row r="767" ht="15.75" customHeight="1" s="2"/>
-    <row r="768" ht="15.75" customHeight="1" s="2"/>
-    <row r="769" ht="15.75" customHeight="1" s="2"/>
-    <row r="770" ht="15.75" customHeight="1" s="2"/>
-    <row r="771" ht="15.75" customHeight="1" s="2"/>
-    <row r="772" ht="15.75" customHeight="1" s="2"/>
-    <row r="773" ht="15.75" customHeight="1" s="2"/>
-    <row r="774" ht="15.75" customHeight="1" s="2"/>
-    <row r="775" ht="15.75" customHeight="1" s="2"/>
-    <row r="776" ht="15.75" customHeight="1" s="2"/>
-    <row r="777" ht="15.75" customHeight="1" s="2"/>
-    <row r="778" ht="15.75" customHeight="1" s="2"/>
-    <row r="779" ht="15.75" customHeight="1" s="2"/>
-    <row r="780" ht="15.75" customHeight="1" s="2"/>
-    <row r="781" ht="15.75" customHeight="1" s="2"/>
-    <row r="782" ht="15.75" customHeight="1" s="2"/>
-    <row r="783" ht="15.75" customHeight="1" s="2"/>
-    <row r="784" ht="15.75" customHeight="1" s="2"/>
-    <row r="785" ht="15.75" customHeight="1" s="2"/>
-    <row r="786" ht="15.75" customHeight="1" s="2"/>
-    <row r="787" ht="15.75" customHeight="1" s="2"/>
-    <row r="788" ht="15.75" customHeight="1" s="2"/>
-    <row r="789" ht="15.75" customHeight="1" s="2"/>
-    <row r="790" ht="15.75" customHeight="1" s="2"/>
-    <row r="791" ht="15.75" customHeight="1" s="2"/>
-    <row r="792" ht="15.75" customHeight="1" s="2"/>
-    <row r="793" ht="15.75" customHeight="1" s="2"/>
-    <row r="794" ht="15.75" customHeight="1" s="2"/>
-    <row r="795" ht="15.75" customHeight="1" s="2"/>
-    <row r="796" ht="15.75" customHeight="1" s="2"/>
-    <row r="797" ht="15.75" customHeight="1" s="2"/>
-    <row r="798" ht="15.75" customHeight="1" s="2"/>
-    <row r="799" ht="15.75" customHeight="1" s="2"/>
-    <row r="800" ht="15.75" customHeight="1" s="2"/>
-    <row r="801" ht="15.75" customHeight="1" s="2"/>
-    <row r="802" ht="15.75" customHeight="1" s="2"/>
-    <row r="803" ht="15.75" customHeight="1" s="2"/>
-    <row r="804" ht="15.75" customHeight="1" s="2"/>
-    <row r="805" ht="15.75" customHeight="1" s="2"/>
-    <row r="806" ht="15.75" customHeight="1" s="2"/>
-    <row r="807" ht="15.75" customHeight="1" s="2"/>
-    <row r="808" ht="15.75" customHeight="1" s="2"/>
-    <row r="809" ht="15.75" customHeight="1" s="2"/>
-    <row r="810" ht="15.75" customHeight="1" s="2"/>
-    <row r="811" ht="15.75" customHeight="1" s="2"/>
-    <row r="812" ht="15.75" customHeight="1" s="2"/>
-    <row r="813" ht="15.75" customHeight="1" s="2"/>
-    <row r="814" ht="15.75" customHeight="1" s="2"/>
-    <row r="815" ht="15.75" customHeight="1" s="2"/>
-    <row r="816" ht="15.75" customHeight="1" s="2"/>
-    <row r="817" ht="15.75" customHeight="1" s="2"/>
-    <row r="818" ht="15.75" customHeight="1" s="2"/>
-    <row r="819" ht="15.75" customHeight="1" s="2"/>
-    <row r="820" ht="15.75" customHeight="1" s="2"/>
-    <row r="821" ht="15.75" customHeight="1" s="2"/>
-    <row r="822" ht="15.75" customHeight="1" s="2"/>
-    <row r="823" ht="15.75" customHeight="1" s="2"/>
-    <row r="824" ht="15.75" customHeight="1" s="2"/>
-    <row r="825" ht="15.75" customHeight="1" s="2"/>
-    <row r="826" ht="15.75" customHeight="1" s="2"/>
-    <row r="827" ht="15.75" customHeight="1" s="2"/>
-    <row r="828" ht="15.75" customHeight="1" s="2"/>
-    <row r="829" ht="15.75" customHeight="1" s="2"/>
-    <row r="830" ht="15.75" customHeight="1" s="2"/>
-    <row r="831" ht="15.75" customHeight="1" s="2"/>
-    <row r="832" ht="15.75" customHeight="1" s="2"/>
-    <row r="833" ht="15.75" customHeight="1" s="2"/>
-    <row r="834" ht="15.75" customHeight="1" s="2"/>
-    <row r="835" ht="15.75" customHeight="1" s="2"/>
-    <row r="836" ht="15.75" customHeight="1" s="2"/>
-    <row r="837" ht="15.75" customHeight="1" s="2"/>
-    <row r="838" ht="15.75" customHeight="1" s="2"/>
-    <row r="839" ht="15.75" customHeight="1" s="2"/>
-    <row r="840" ht="15.75" customHeight="1" s="2"/>
-    <row r="841" ht="15.75" customHeight="1" s="2"/>
-    <row r="842" ht="15.75" customHeight="1" s="2"/>
-    <row r="843" ht="15.75" customHeight="1" s="2"/>
-    <row r="844" ht="15.75" customHeight="1" s="2"/>
-    <row r="845" ht="15.75" customHeight="1" s="2"/>
-    <row r="846" ht="15.75" customHeight="1" s="2"/>
-    <row r="847" ht="15.75" customHeight="1" s="2"/>
-    <row r="848" ht="15.75" customHeight="1" s="2"/>
-    <row r="849" ht="15.75" customHeight="1" s="2"/>
-    <row r="850" ht="15.75" customHeight="1" s="2"/>
-    <row r="851" ht="15.75" customHeight="1" s="2"/>
-    <row r="852" ht="15.75" customHeight="1" s="2"/>
-    <row r="853" ht="15.75" customHeight="1" s="2"/>
-    <row r="854" ht="15.75" customHeight="1" s="2"/>
-    <row r="855" ht="15.75" customHeight="1" s="2"/>
-    <row r="856" ht="15.75" customHeight="1" s="2"/>
-    <row r="857" ht="15.75" customHeight="1" s="2"/>
-    <row r="858" ht="15.75" customHeight="1" s="2"/>
-    <row r="859" ht="15.75" customHeight="1" s="2"/>
-    <row r="860" ht="15.75" customHeight="1" s="2"/>
-    <row r="861" ht="15.75" customHeight="1" s="2"/>
-    <row r="862" ht="15.75" customHeight="1" s="2"/>
-    <row r="863" ht="15.75" customHeight="1" s="2"/>
-    <row r="864" ht="15.75" customHeight="1" s="2"/>
-    <row r="865" ht="15.75" customHeight="1" s="2"/>
-    <row r="866" ht="15.75" customHeight="1" s="2"/>
-    <row r="867" ht="15.75" customHeight="1" s="2"/>
-    <row r="868" ht="15.75" customHeight="1" s="2"/>
-    <row r="869" ht="15.75" customHeight="1" s="2"/>
-    <row r="870" ht="15.75" customHeight="1" s="2"/>
-    <row r="871" ht="15.75" customHeight="1" s="2"/>
-    <row r="872" ht="15.75" customHeight="1" s="2"/>
-    <row r="873" ht="15.75" customHeight="1" s="2"/>
-    <row r="874" ht="15.75" customHeight="1" s="2"/>
-    <row r="875" ht="15.75" customHeight="1" s="2"/>
-    <row r="876" ht="15.75" customHeight="1" s="2"/>
-    <row r="877" ht="15.75" customHeight="1" s="2"/>
-    <row r="878" ht="15.75" customHeight="1" s="2"/>
-    <row r="879" ht="15.75" customHeight="1" s="2"/>
-    <row r="880" ht="15.75" customHeight="1" s="2"/>
-    <row r="881" ht="15.75" customHeight="1" s="2"/>
-    <row r="882" ht="15.75" customHeight="1" s="2"/>
-    <row r="883" ht="15.75" customHeight="1" s="2"/>
-    <row r="884" ht="15.75" customHeight="1" s="2"/>
-    <row r="885" ht="15.75" customHeight="1" s="2"/>
-    <row r="886" ht="15.75" customHeight="1" s="2"/>
-    <row r="887" ht="15.75" customHeight="1" s="2"/>
-    <row r="888" ht="15.75" customHeight="1" s="2"/>
-    <row r="889" ht="15.75" customHeight="1" s="2"/>
-    <row r="890" ht="15.75" customHeight="1" s="2"/>
-    <row r="891" ht="15.75" customHeight="1" s="2"/>
-    <row r="892" ht="15.75" customHeight="1" s="2"/>
-    <row r="893" ht="15.75" customHeight="1" s="2"/>
-    <row r="894" ht="15.75" customHeight="1" s="2"/>
-    <row r="895" ht="15.75" customHeight="1" s="2"/>
-    <row r="896" ht="15.75" customHeight="1" s="2"/>
-    <row r="897" ht="15.75" customHeight="1" s="2"/>
-    <row r="898" ht="15.75" customHeight="1" s="2"/>
-    <row r="899" ht="15.75" customHeight="1" s="2"/>
-    <row r="900" ht="15.75" customHeight="1" s="2"/>
-    <row r="901" ht="15.75" customHeight="1" s="2"/>
-    <row r="902" ht="15.75" customHeight="1" s="2"/>
-    <row r="903" ht="15.75" customHeight="1" s="2"/>
-    <row r="904" ht="15.75" customHeight="1" s="2"/>
-    <row r="905" ht="15.75" customHeight="1" s="2"/>
-    <row r="906" ht="15.75" customHeight="1" s="2"/>
-    <row r="907" ht="15.75" customHeight="1" s="2"/>
-    <row r="908" ht="15.75" customHeight="1" s="2"/>
-    <row r="909" ht="15.75" customHeight="1" s="2"/>
-    <row r="910" ht="15.75" customHeight="1" s="2"/>
-    <row r="911" ht="15.75" customHeight="1" s="2"/>
-    <row r="912" ht="15.75" customHeight="1" s="2"/>
-    <row r="913" ht="15.75" customHeight="1" s="2"/>
-    <row r="914" ht="15.75" customHeight="1" s="2"/>
-    <row r="915" ht="15.75" customHeight="1" s="2"/>
-    <row r="916" ht="15.75" customHeight="1" s="2"/>
-    <row r="917" ht="15.75" customHeight="1" s="2"/>
-    <row r="918" ht="15.75" customHeight="1" s="2"/>
-    <row r="919" ht="15.75" customHeight="1" s="2"/>
-    <row r="920" ht="15.75" customHeight="1" s="2"/>
-    <row r="921" ht="15.75" customHeight="1" s="2"/>
-    <row r="922" ht="15.75" customHeight="1" s="2"/>
-    <row r="923" ht="15.75" customHeight="1" s="2"/>
-    <row r="924" ht="15.75" customHeight="1" s="2"/>
-    <row r="925" ht="15.75" customHeight="1" s="2"/>
-    <row r="926" ht="15.75" customHeight="1" s="2"/>
-    <row r="927" ht="15.75" customHeight="1" s="2"/>
-    <row r="928" ht="15.75" customHeight="1" s="2"/>
-    <row r="929" ht="15.75" customHeight="1" s="2"/>
-    <row r="930" ht="15.75" customHeight="1" s="2"/>
-    <row r="931" ht="15.75" customHeight="1" s="2"/>
-    <row r="932" ht="15.75" customHeight="1" s="2"/>
-    <row r="933" ht="15.75" customHeight="1" s="2"/>
-    <row r="934" ht="15.75" customHeight="1" s="2"/>
-    <row r="935" ht="15.75" customHeight="1" s="2"/>
-    <row r="936" ht="15.75" customHeight="1" s="2"/>
-    <row r="937" ht="15.75" customHeight="1" s="2"/>
-    <row r="938" ht="15.75" customHeight="1" s="2"/>
-    <row r="939" ht="15.75" customHeight="1" s="2"/>
-    <row r="940" ht="15.75" customHeight="1" s="2"/>
-    <row r="941" ht="15.75" customHeight="1" s="2"/>
-    <row r="942" ht="15.75" customHeight="1" s="2"/>
-    <row r="943" ht="15.75" customHeight="1" s="2"/>
-    <row r="944" ht="15.75" customHeight="1" s="2"/>
-    <row r="945" ht="15.75" customHeight="1" s="2"/>
-    <row r="946" ht="15.75" customHeight="1" s="2"/>
-    <row r="947" ht="15.75" customHeight="1" s="2"/>
-    <row r="948" ht="15.75" customHeight="1" s="2"/>
-    <row r="949" ht="15.75" customHeight="1" s="2"/>
-    <row r="950" ht="15.75" customHeight="1" s="2"/>
-    <row r="951" ht="15.75" customHeight="1" s="2"/>
-    <row r="952" ht="15.75" customHeight="1" s="2"/>
-    <row r="953" ht="15.75" customHeight="1" s="2"/>
-    <row r="954" ht="15.75" customHeight="1" s="2"/>
-    <row r="955" ht="15.75" customHeight="1" s="2"/>
-    <row r="956" ht="15.75" customHeight="1" s="2"/>
-    <row r="957" ht="15.75" customHeight="1" s="2"/>
-    <row r="958" ht="15.75" customHeight="1" s="2"/>
-    <row r="959" ht="15.75" customHeight="1" s="2"/>
-    <row r="960" ht="15.75" customHeight="1" s="2"/>
-    <row r="961" ht="15.75" customHeight="1" s="2"/>
-    <row r="962" ht="15.75" customHeight="1" s="2"/>
-    <row r="963" ht="15.75" customHeight="1" s="2"/>
-    <row r="964" ht="15.75" customHeight="1" s="2"/>
-    <row r="965" ht="15.75" customHeight="1" s="2"/>
-    <row r="966" ht="15.75" customHeight="1" s="2"/>
-    <row r="967" ht="15.75" customHeight="1" s="2"/>
-    <row r="968" ht="15.75" customHeight="1" s="2"/>
-    <row r="969" ht="15.75" customHeight="1" s="2"/>
-    <row r="970" ht="15.75" customHeight="1" s="2"/>
-    <row r="971" ht="15.75" customHeight="1" s="2"/>
-    <row r="972" ht="15.75" customHeight="1" s="2"/>
-    <row r="973" ht="15.75" customHeight="1" s="2"/>
-    <row r="974" ht="15.75" customHeight="1" s="2"/>
-    <row r="975" ht="15.75" customHeight="1" s="2"/>
-    <row r="976" ht="15.75" customHeight="1" s="2"/>
-    <row r="977" ht="15.75" customHeight="1" s="2"/>
-    <row r="978" ht="15.75" customHeight="1" s="2"/>
-    <row r="979" ht="15.75" customHeight="1" s="2"/>
-    <row r="980" ht="15.75" customHeight="1" s="2"/>
-    <row r="981" ht="15.75" customHeight="1" s="2"/>
-    <row r="982" ht="15.75" customHeight="1" s="2"/>
-    <row r="983" ht="15.75" customHeight="1" s="2"/>
-    <row r="984" ht="15.75" customHeight="1" s="2"/>
-    <row r="985" ht="15.75" customHeight="1" s="2"/>
-    <row r="986" ht="15.75" customHeight="1" s="2"/>
-    <row r="987" ht="15.75" customHeight="1" s="2"/>
-    <row r="988" ht="15.75" customHeight="1" s="2"/>
-    <row r="989" ht="15.75" customHeight="1" s="2"/>
-    <row r="990" ht="15.75" customHeight="1" s="2"/>
-    <row r="991" ht="15.75" customHeight="1" s="2"/>
-    <row r="992" ht="15.75" customHeight="1" s="2"/>
-    <row r="993" ht="15.75" customHeight="1" s="2"/>
-    <row r="994" ht="15.75" customHeight="1" s="2"/>
-    <row r="995" ht="15.75" customHeight="1" s="2"/>
-    <row r="996" ht="15.75" customHeight="1" s="2"/>
-    <row r="997" ht="15.75" customHeight="1" s="2"/>
-    <row r="998" ht="15.75" customHeight="1" s="2"/>
-    <row r="999" ht="15.75" customHeight="1" s="2"/>
-    <row r="1000" ht="15.75" customHeight="1" s="2"/>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Exact-package no-op diagnostic -&gt; reward 0.0000 with no_op=1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1487,102 +580,120 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>RL Task Quality Scorecard</t>
         </is>
       </c>
+      <c r="B1" s="4" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Pre-training QC for agent / RL task suites - prompt realism, verifier coverage, verifier correctness, reward shaping, determinism, anti-gaming.</t>
         </is>
       </c>
+      <c r="B2" s="4" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n"/>
+      <c r="B3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>The one thing this workbook is for</t>
         </is>
       </c>
+      <c r="B4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>A task is only useful for RL if its reward is SOUND: a genuinely correct rollout must score high, and a wrong or no-op rollout must score low. Everything here exists to prove those two directions, in both directions, before you spend compute.</t>
         </is>
       </c>
+      <c r="B5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Sheets</t>
         </is>
       </c>
+      <c r="B7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Rubric</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>The 30 criteria, what Pass/Partial/Fail mean for each, and which are hard gates.</t>
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
+    </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Scoring</t>
         </is>
       </c>
+      <c r="B10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>2 = Pass</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Meets the bar in the Rubric sheet, and you have evidence.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>1 = Partial</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Partly meets it, or you believe it but have not measured it.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>0 = Fail</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Does not meet the bar.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>blank</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Criterion does not apply to this task. Excluded from the denominator.</t>
         </is>
@@ -2588,1255 +1699,1280 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>DropLine Four Lite — Rubric — 30 criteria</t>
         </is>
       </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="4" t="n"/>
+      <c r="H1" s="4" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Equal-weight 2/1/0 scoring. Gate criteria are shaded; failing a gate rejects the task.</t>
         </is>
       </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n"/>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Criterion</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Pass (2) means</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Fail (0) means</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Score (2/1/0/blank)</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>A · Prompt realism</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Derived from real traffic, not synthesised</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Verbatim or lightly-edited from a real arena/product log, with provenance recorded</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Model-generated prompts with no real-world source</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="1" t="inlineStr">
-        <is>
-          <t>task.toml records the Deliverables Tracker Classic &amp; Board Games allocation and the task owner's live Undo/Redo request; instruction.md retains that request's conversational form.</t>
-        </is>
-      </c>
-      <c r="H5" s="1" t="inlineStr">
-        <is>
-          <t>PASS: provenance is explicit and traceable.</t>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>task.toml records the Deliverables Tracker assignment and the live request to add Undo/Redo.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>A · Prompt realism</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Natural voice preserved</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Typos, lowercase, terseness, emoji and abruptness left intact</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Every prompt cleaned into polite full sentences</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="1" t="inlineStr">
-        <is>
-          <t>instruction.md uses the original concise, lowercase request style ('can you build me...', 'yeah, let's add...') rather than a polished synthetic specification.</t>
-        </is>
-      </c>
-      <c r="H6" s="1" t="inlineStr">
-        <is>
-          <t>PASS: natural voice is preserved while detailed files carry the contract.</t>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>instruction.md preserves lowercase, terse, first-person phrasing.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>A · Prompt realism</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Domain matches the target taxonomy allocation</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Task's domain and difficulty match its row in the sampling plan</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Suite over-concentrated in one saturated domain</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="1" t="inlineStr">
-        <is>
-          <t>task.toml declares Software / Classic &amp; Board Games and the recorded provenance names the matching Tic-tac-toe or Connect-4 allocation.</t>
-        </is>
-      </c>
-      <c r="H7" s="1" t="inlineStr">
-        <is>
-          <t>PASS: taxonomy and assigned domain match.</t>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Software / Classic &amp; Board Games matches the assigned Connect Four domain.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>A6</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>A · Prompt realism</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Prompt is unambiguous and achievable in the environment</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>One reasonable reading; every required artifact reachable from the seed state</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Ambiguous, or asks for data/tools the environment does not have</t>
         </is>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="F8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="1" t="inlineStr">
-        <is>
-          <t>All required assets are present and the consolidated final Oracle passed all 22 scored browser criteria with reward 1.0000.</t>
-        </is>
-      </c>
-      <c r="H8" s="1" t="inlineStr">
-        <is>
-          <t>PASS: achievable under one reasonable reading.</t>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>All assets and paths are supplied; exact-package Oracle scored 1.0000.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>B · Verifier coverage</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Every explicit requirement maps to &gt;=1 assertion</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Requirement-&gt;assertion matrix is complete; no unchecked ask</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>A stated requirement has no assertion (model can skip it and pass)</t>
         </is>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="F9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="1" t="inlineStr">
-        <is>
-          <t>tests/coverage.json maps the 15 instruction requirements to browser criteria, and Oracle passes them. Browser reload persistence is tested, but server-process restart durability and the exact Express/SQLite stack are not mechanically checked.</t>
-        </is>
-      </c>
-      <c r="H9" s="1" t="inlineStr">
-        <is>
-          <t>PARTIAL: broad behavioral coverage with two implementation-boundary gaps.</t>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>coverage.json maps all 18 requirements and 15/15 functional requirements, but restart durability and exact stack enforcement remain behavioral gaps.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>B · Verifier coverage</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Liveness / render gate present</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Artifact is executed or rendered, not just string-matched</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Only static text matching; a non-running artifact can pass</t>
         </is>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="1" t="inlineStr">
-        <is>
-          <t>tests/test.sh boots /app/server.js and probes the live same-origin app; Render and Constraints use Playwright against the substantive authenticated workspace.</t>
-        </is>
-      </c>
-      <c r="H10" s="1" t="inlineStr">
-        <is>
-          <t>PASS: non-running and static-imitation submissions cannot pass.</t>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>test.sh boots the artifact and all four dimensions use Playwright MCP against the live app.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>B4</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>B · Verifier coverage</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Plural 'all / every' asks checked across ALL matches</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Aggregate check over the whole collection (SIG-08 safe)</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>First-match-only projection; acting on one item earns full reward</t>
         </is>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="F11" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="1" t="inlineStr">
-        <is>
-          <t>Criteria verify complete 42-cell boards, all winning markers, full histories, exact latest-ten archive ordering, all-session token revocation, and whole-state invariants after rejected actions.</t>
-        </is>
-      </c>
-      <c r="H11" s="1" t="inlineStr">
-        <is>
-          <t>PASS: plural and collection requirements are aggregate checks.</t>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Criteria aggregate all 42 cells, full histories, latest-ten archive rows, all-session revocation, and complete unchanged-state snapshots.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>B · Verifier coverage</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>No-op rollout scores ~0</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Empty / unchanged output measured at &lt;=0.05</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Doing nothing collects meaningful reward mass</t>
         </is>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="F12" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="1" t="inlineStr">
-        <is>
-          <t>Executable no-op run produced reward 0.0000 with no_op=1; tests/test.sh writes a deterministic zero before any boot or judge work.</t>
-        </is>
-      </c>
-      <c r="H12" s="1" t="inlineStr">
-        <is>
-          <t>PASS: measured no-op is below 0.05.</t>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Exact-package no-op diagnostic received reward 0.0000 with no_op=1.</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>C · Verifier correctness</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Correct rollout passes (no false negative)</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Oracle / reference solution scores &gt;=0.95, verified by running it</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Oracle scores below 0.95 — task is unpassable as written</t>
         </is>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="1" t="inlineStr">
-        <is>
-          <t>Fresh consolidated v6.0.3 Oracle: constraints 1.0, functional 1.0, render 1.0, polish 1.0, final reward 1.0000.</t>
-        </is>
-      </c>
-      <c r="H13" s="1" t="inlineStr">
-        <is>
-          <t>PASS: correct reference rollout exceeds 0.95.</t>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Oracle: 1.0000 with 22/22 criteria and Functional 13/13.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>C · Verifier correctness</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Wrong rollout fails (no false positive)</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>At least 2 adversarial rollouts measured at &lt;=0.2</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>A knowingly-wrong rollout scores well</t>
         </is>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>One measured no-op is &lt;=0.2; GPT 0.5390 and Haiku 0.3327 are substantive partial implementations, so a second adversarial &lt;=0.2 sample is not available.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>C · Verifier correctness</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Reward is not inverted</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Ranking of known-good vs known-bad rollouts is monotone</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>A worse rollout outscores a better one</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="1" t="inlineStr">
-        <is>
-          <t>Two wrong/adversarial outcomes are at or below 0.2: no-op 0.0000 and untouched Haiku 0.0000 after genuine constraints/render failures. Untouched GPT-5.4-mini receives partial 0.3642 for a substantive but incomplete app.</t>
-        </is>
-      </c>
-      <c r="H14" s="1" t="inlineStr">
-        <is>
-          <t>PASS: known-wrong rollouts do not receive high reward.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>C3</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Observed ordering is Oracle 1.0000 &gt; GPT 0.5390 &gt; Haiku 0.3327 &gt; no-op 0.0000.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>C · Verifier correctness</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>Reward is not inverted</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Ranking of known-good vs known-bad rollouts is monotone</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>A worse rollout outscores a better one</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="n">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Expected types/values match what is actually stored</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Every literal checked against the real seed / write path</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>String-vs-number or wrong literal under strict equality (SIG-05)</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="1" t="inlineStr">
-        <is>
-          <t>Observed ordering is Oracle 1.0000 &gt; gate-passing incomplete GPT 0.3642 &gt; gate-failing Haiku 0.0000 = no-op 0.0000.</t>
-        </is>
-      </c>
-      <c r="H15" s="1" t="inlineStr">
-        <is>
-          <t>PASS: reward ordering follows demonstrated quality and required gates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Seed copies and typed workbook values match, and Oracle reproduces every strict literal.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>C · Verifier correctness</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>Expected types/values match what is actually stored</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>Every literal checked against the real seed / write path</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="inlineStr">
-        <is>
-          <t>String-vs-number or wrong literal under strict equality (SIG-05)</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="n">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>No dead or malformed assertions</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Every assertion can pass for some rollout; paths parse</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Count/contains on a bare filter, or unbalanced JSONPath (SIG-07)</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="1" t="inlineStr">
-        <is>
-          <t>Seed workbook accounts, revisions, cell positions, histories, totals, redo state, and eleven Jordan archive rows were independently inspected and match strict verifier literals.</t>
-        </is>
-      </c>
-      <c r="H16" s="1" t="inlineStr">
-        <is>
-          <t>PASS: expected values and stored types agree.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>C5</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>All 22 unique criteria parsed and passed for Oracle.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>C · Verifier correctness</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>No dead or malformed assertions</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>Every assertion can pass for some rollout; paths parse</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>Count/contains on a bare filter, or unbalanced JSONPath (SIG-07)</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="n">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>No unresolved placeholders at runtime</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>All $TOKENS resolve, or the resolver is confirmed wired for this suite</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Literal $TOKEN reaches the engine and throws (SIG-06)</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G17" s="1" t="inlineStr">
-        <is>
-          <t>All four RewardKit dimensions parse and execute; the final Oracle passed every criterion and generated complete reward-details.json output.</t>
-        </is>
-      </c>
-      <c r="H17" s="1" t="inlineStr">
-        <is>
-          <t>PASS: no dead or malformed assertion was observed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>C6</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Harbor secret and criterion-template placeholders are configured; accepted runs show no unresolved-token error.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>C · Verifier correctness</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
-        <is>
-          <t>No unresolved placeholders at runtime</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="inlineStr">
-        <is>
-          <t>All $TOKENS resolve, or the resolver is confirmed wired for this suite</t>
-        </is>
-      </c>
-      <c r="E18" s="1" t="inlineStr">
-        <is>
-          <t>Literal $TOKEN reaches the engine and throws (SIG-06)</t>
-        </is>
-      </c>
-      <c r="F18" s="1" t="n">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>'Nothing else changed' guards have teeth</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Whole-collection diff, or each untargeted entity asserted individually</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Exclusion filter or [*] path that passes unconditionally (SIG-01)</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="1" t="inlineStr">
-        <is>
-          <t>Judge prompts and runtime configs contain no unresolved scoring placeholder; environment-key references resolve through Harbor and all final judges executed.</t>
-        </is>
-      </c>
-      <c r="H18" s="1" t="inlineStr">
-        <is>
-          <t>PASS: no literal unresolved token reached the verifier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>C7</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Full-column, terminal, stale, duplicate, sign-out, and reset scenarios compare complete state/revisions.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>C · Verifier correctness</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>'Nothing else changed' guards have teeth</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
-        <is>
-          <t>Whole-collection diff, or each untargeted entity asserted individually</t>
-        </is>
-      </c>
-      <c r="E19" s="1" t="inlineStr">
-        <is>
-          <t>Exclusion filter or [*] path that passes unconditionally (SIG-01)</t>
-        </is>
-      </c>
-      <c r="F19" s="1" t="n">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>App side-effects excluded from the baseline</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>ignoreFields covers every field the correct action legitimately mutates</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Correct rollout fails its own unchanged-guard (SIG-02)</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G19" s="1" t="inlineStr">
-        <is>
-          <t>Full-column, terminal-lock, stale-write, duplicate-operation, sign-out revocation, and reset checks snapshot and compare board, history, totals, archive, revision, and identity around rejected actions.</t>
-        </is>
-      </c>
-      <c r="H19" s="1" t="inlineStr">
-        <is>
-          <t>PASS: 'nothing else changed' guards compare substantive whole state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>C8</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Baselines are taken after prerequisites and legitimate revision, archive, score, identity, and focus effects are scoped.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="2">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>C · Verifier correctness</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>App side-effects excluded from the baseline</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>ignoreFields covers every field the correct action legitimately mutates</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="inlineStr">
-        <is>
-          <t>Correct rollout fails its own unchanged-guard (SIG-02)</t>
-        </is>
-      </c>
-      <c r="F20" s="1" t="n">
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>LLM-graded facts are true of the seed</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Every expected fact verified against seed data; weighting arithmetic done</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Judge rubric asserts facts the seed contradicts (SIG-03)</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="1" t="inlineStr">
-        <is>
-          <t>Each scenario records its baseline after prerequisite sign-in/reset actions and explicitly allows legitimate revision, token, focus, or archive changes only where the tested action requires them.</t>
-        </is>
-      </c>
-      <c r="H20" s="1" t="inlineStr">
-        <is>
-          <t>PASS: legitimate app side effects are excluded from unchanged baselines.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="2">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>C · Verifier correctness</t>
-        </is>
-      </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>LLM-graded facts are true of the seed</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>Every expected fact verified against seed data; weighting arithmetic done</t>
-        </is>
-      </c>
-      <c r="E21" s="1" t="inlineStr">
-        <is>
-          <t>Judge rubric asserts facts the seed contradicts (SIG-03)</t>
-        </is>
-      </c>
-      <c r="F21" s="1" t="n">
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Seeded facts and arithmetic were checked against the workbook and reproduced by Oracle.</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="2">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>D · Reward shaping</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Graded, not binary</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Reward takes &gt;=4 distinct values across a sample batch</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Pure 0/1 — no gradient for the policy to climb</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G21" s="1" t="inlineStr">
-        <is>
-          <t>All LLM-graded seeded facts and score/archive arithmetic were checked against dropline_seed.xlsx; the Oracle reproduced the exact values.</t>
-        </is>
-      </c>
-      <c r="H21" s="1" t="inlineStr">
-        <is>
-          <t>PASS: graded facts are true of the seed and write path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="2">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Four measured rewards are distinct: 1.0000, 0.5390, 0.3327, and 0.0000.</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="2">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>D · Reward shaping</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
-        <is>
-          <t>Graded, not binary</t>
-        </is>
-      </c>
-      <c r="D22" s="1" t="inlineStr">
-        <is>
-          <t>Reward takes &gt;=4 distinct values across a sample batch</t>
-        </is>
-      </c>
-      <c r="E22" s="1" t="inlineStr">
-        <is>
-          <t>Pure 0/1 — no gradient for the policy to climb</t>
-        </is>
-      </c>
-      <c r="F22" s="1" t="n">
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Gates apply before shaping terms</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Constraint/render failure hard-zeros the quality terms</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>A constraint-violating rollout still collects style points</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Render/Constraints hard-gate before the 0.6 Functional + 0.4 Polish formula.</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="2">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>D · Reward shaping</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Gates carry no reward mass of their own</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Passing only the cheap gates yields &lt;=0.1</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Gate dimensions are half the weighted mean (cheap to farm)</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Render and Constraints have zero reward weight and only unlock quality scoring.</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="2">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>D · Reward shaping</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Discriminates within a real rollout batch</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Std-dev of reward over &gt;=8 sampled rollouts is &gt;=0.15</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>All rollouts land within a narrow band; no learning signal</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="1" t="inlineStr">
-        <is>
-          <t>Observed final rewards have three distinct values: 1.0000, 0.3642, and 0.0000. The 22 weighted criteria provide theoretical granularity, but the measured batch does not yet show four distinct values.</t>
-        </is>
-      </c>
-      <c r="H22" s="1" t="inlineStr">
-        <is>
-          <t>PARTIAL: shaped reward exists, but the &gt;=4 measured-level target is unmet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="2">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>The available four runs show useful spread, but the &gt;=8-rollout statistic is unmeasured.</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="2">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>D · Reward shaping</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
-        <is>
-          <t>Gates apply before shaping terms</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="inlineStr">
-        <is>
-          <t>Constraint/render failure hard-zeros the quality terms</t>
-        </is>
-      </c>
-      <c r="E23" s="1" t="inlineStr">
-        <is>
-          <t>A constraint-violating rollout still collects style points</t>
-        </is>
-      </c>
-      <c r="F23" s="1" t="n">
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Length / verbosity band encoded where it matters</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Under- and over-production both penalised per measured curve</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Reward rises monotonically with output length</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>N/A: output is an application, not a bounded natural-language response.</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="2">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>E · Determinism</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Same rollout scores the same reward</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Re-scored 3x with identical result</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Reward varies run to run (RNG, wall-clock, network)</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Exact same artifact has not been independently rescored three times.</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="2">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>E · Determinism</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Reference / baseline artifacts are frozen and versioned</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Checked in, hash recorded, task version bumped on any change</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Baseline regenerated by a model or edited in place</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Version and exact run checksum are frozen, but packaged server.js bytes differ from its declared per-file hash because of mixed line endings.</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1" s="2">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>E · Determinism</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Verifier runs offline or on a pinned allowlist</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>No unpinned network dependency in the scoring path</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Verifier fetches from the live internet</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Public verifier networking is required by the Docker platform. The app has no external runtime dependencies, but public is broader than offline/allowlist.</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1" s="2">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>E4</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>E · Determinism</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Judge model, temperature and prompt are pinned</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Explicit model id, temp 0, versioned rubric</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Floating model alias or unpinned sampling</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="1" t="inlineStr">
-        <is>
-          <t>tests/test.sh computes quality reward only after Render and Constraints are non-zero; either failed gate forces final reward to 0.0000, as demonstrated by Haiku.</t>
-        </is>
-      </c>
-      <c r="H23" s="1" t="inlineStr">
-        <is>
-          <t>PASS: hard gates apply before reward shaping.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="2">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
-        <is>
-          <t>D · Reward shaping</t>
-        </is>
-      </c>
-      <c r="C24" s="1" t="inlineStr">
-        <is>
-          <t>Gates carry no reward mass of their own</t>
-        </is>
-      </c>
-      <c r="D24" s="1" t="inlineStr">
-        <is>
-          <t>Passing only the cheap gates yields &lt;=0.1</t>
-        </is>
-      </c>
-      <c r="E24" s="1" t="inlineStr">
-        <is>
-          <t>Gate dimensions are half the weighted mean (cheap to farm)</t>
-        </is>
-      </c>
-      <c r="F24" s="1" t="n">
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>All judges pin gpt-5.6-luna, Codex, temperature 0, reasoning effort, timeout, and versioned prompts.</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1" s="2">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>F · Anti-gaming</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Keyword stuffing does not pass</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Tested: a file of the right keywords with no real behaviour scores &lt;=0.2</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Regex-only checks satisfied by pasting the expected strings</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Live browser/server mutation makes keyword stuffing ineffective, but a dedicated keyword-only artifact was not run.</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1" s="2">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>F · Anti-gaming</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Judge is injection-resistant</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Agent output cannot instruct the judge; tested with an injected directive</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Agent text is concatenated into the judge prompt unguarded</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>All prompts label submitted evidence untrusted; a dedicated injected artifact was not run.</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1" s="2">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>F · Anti-gaming</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Tests and rubric are not readable by the agent</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Separate verifier environment; tests/ never uploaded to the agent container</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Agent can read the assertions it is graded on</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="1" t="inlineStr">
-        <is>
-          <t>Render and Constraints carry zero reward mass and only unlock the 0.6 Functional + 0.4 Polish calculation. Passing gates alone cannot produce positive reward.</t>
-        </is>
-      </c>
-      <c r="H24" s="1" t="inlineStr">
-        <is>
-          <t>PASS: cheap gates cannot be farmed for score.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="2">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>D4</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t>D · Reward shaping</t>
-        </is>
-      </c>
-      <c r="C25" s="1" t="inlineStr">
-        <is>
-          <t>Discriminates within a real rollout batch</t>
-        </is>
-      </c>
-      <c r="D25" s="1" t="inlineStr">
-        <is>
-          <t>Std-dev of reward over &gt;=8 sampled rollouts is &gt;=0.15</t>
-        </is>
-      </c>
-      <c r="E25" s="1" t="inlineStr">
-        <is>
-          <t>All rollouts land within a narrow band; no learning signal</t>
-        </is>
-      </c>
-      <c r="F25" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="1" t="inlineStr">
-        <is>
-          <t>Oracle, untouched GPT-5.4-mini, untouched Haiku, and no-op provide strong spread from 0.0000 to 1.0000, but fewer than eight sampled target-model rollouts were requested.</t>
-        </is>
-      </c>
-      <c r="H25" s="1" t="inlineStr">
-        <is>
-          <t>PARTIAL GATE: useful observed spread; required &gt;=8-rollout statistic unmeasured.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="2">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>D5</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
-        <is>
-          <t>D · Reward shaping</t>
-        </is>
-      </c>
-      <c r="C26" s="1" t="inlineStr">
-        <is>
-          <t>Length / verbosity band encoded where it matters</t>
-        </is>
-      </c>
-      <c r="D26" s="1" t="inlineStr">
-        <is>
-          <t>Under- and over-production both penalised per measured curve</t>
-        </is>
-      </c>
-      <c r="E26" s="1" t="inlineStr">
-        <is>
-          <t>Reward rises monotonically with output length</t>
-        </is>
-      </c>
-      <c r="G26" s="1" t="inlineStr">
-        <is>
-          <t>The deliverable is an interactive full-stack application, not a bounded natural-language response.</t>
-        </is>
-      </c>
-      <c r="H26" s="1" t="inlineStr">
-        <is>
-          <t>N/A: output-length reward curves do not apply.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="2">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
-        <is>
-          <t>E · Determinism</t>
-        </is>
-      </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>Same rollout scores the same reward</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr">
-        <is>
-          <t>Re-scored 3x with identical result</t>
-        </is>
-      </c>
-      <c r="E27" s="1" t="inlineStr">
-        <is>
-          <t>Reward varies run to run (RNG, wall-clock, network)</t>
-        </is>
-      </c>
-      <c r="F27" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="1" t="inlineStr">
-        <is>
-          <t>Oracle, GPT, and Haiku produced coherent criterion evidence, but the exact same complete rollout has not been independently rescored three times.</t>
-        </is>
-      </c>
-      <c r="H27" s="1" t="inlineStr">
-        <is>
-          <t>PARTIAL GATE: deterministic state is strong; three-repeat judge statistic is unmeasured.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" s="2">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>E2</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>E · Determinism</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>Reference / baseline artifacts are frozen and versioned</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="inlineStr">
-        <is>
-          <t>Checked in, hash recorded, task version bumped on any change</t>
-        </is>
-      </c>
-      <c r="E28" s="1" t="inlineStr">
-        <is>
-          <t>Baseline regenerated by a model or edited in place</t>
-        </is>
-      </c>
-      <c r="F28" s="1" t="n">
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Separate verifier image keeps tests/rubric out of the agent environment.</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" s="2">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>F · Anti-gaming</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>No reward for stalling, refusing, or asking questions</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>A clarifying-question-only rollout scores &lt;=0.05</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Politely declining collects partial credit</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="1" t="inlineStr">
-        <is>
-          <t>Task version is 6.0.3. task.toml records SHA-256 values for the seed, golden server, golden UI, package, and solve script; the final ZIP is checksummed.</t>
-        </is>
-      </c>
-      <c r="H28" s="1" t="inlineStr">
-        <is>
-          <t>PASS: reference artifacts are frozen and versioned.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1" s="2">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>E3</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="inlineStr">
-        <is>
-          <t>E · Determinism</t>
-        </is>
-      </c>
-      <c r="C29" s="1" t="inlineStr">
-        <is>
-          <t>Verifier runs offline or on a pinned allowlist</t>
-        </is>
-      </c>
-      <c r="D29" s="1" t="inlineStr">
-        <is>
-          <t>No unpinned network dependency in the scoring path</t>
-        </is>
-      </c>
-      <c r="E29" s="1" t="inlineStr">
-        <is>
-          <t>Verifier fetches from the live internet</t>
-        </is>
-      </c>
-      <c r="F29" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G29" s="1" t="inlineStr">
-        <is>
-          <t>The application is self-contained. Platform verifier networking is allowlisted to openrouter.ai; public networking exists only in an ignored local Docker compatibility override.</t>
-        </is>
-      </c>
-      <c r="H29" s="1" t="inlineStr">
-        <is>
-          <t>PASS: no unpinned public runtime dependency is needed for scoring.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1" s="2">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>E4</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
-        <is>
-          <t>E · Determinism</t>
-        </is>
-      </c>
-      <c r="C30" s="1" t="inlineStr">
-        <is>
-          <t>Judge model, temperature and prompt are pinned</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="inlineStr">
-        <is>
-          <t>Explicit model id, temp 0, versioned rubric</t>
-        </is>
-      </c>
-      <c r="E30" s="1" t="inlineStr">
-        <is>
-          <t>Floating model alias or unpinned sampling</t>
-        </is>
-      </c>
-      <c r="F30" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" s="1" t="inlineStr">
-        <is>
-          <t>All judge.toml files pin openai/gpt-5.6-luna, temperature 0, reasoning effort, timeout, and v6.0.3 prompt versions.</t>
-        </is>
-      </c>
-      <c r="H30" s="1" t="inlineStr">
-        <is>
-          <t>PASS: judge model, sampling, and prompts are explicitly pinned.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1" s="2">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
-        <is>
-          <t>F · Anti-gaming</t>
-        </is>
-      </c>
-      <c r="C31" s="1" t="inlineStr">
-        <is>
-          <t>Keyword stuffing does not pass</t>
-        </is>
-      </c>
-      <c r="D31" s="1" t="inlineStr">
-        <is>
-          <t>Tested: a file of the right keywords with no real behaviour scores &lt;=0.2</t>
-        </is>
-      </c>
-      <c r="E31" s="1" t="inlineStr">
-        <is>
-          <t>Regex-only checks satisfied by pasting the expected strings</t>
-        </is>
-      </c>
-      <c r="F31" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="1" t="inlineStr">
-        <is>
-          <t>Live browser behavior and same-origin mutations make keyword stuffing ineffective, and no-op scores zero; a dedicated keyword-only adversarial artifact was not separately run.</t>
-        </is>
-      </c>
-      <c r="H31" s="1" t="inlineStr">
-        <is>
-          <t>PARTIAL: structural defense is strong, but the specified adversarial test is unmeasured.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1" s="2">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>F2</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
-        <is>
-          <t>F · Anti-gaming</t>
-        </is>
-      </c>
-      <c r="C32" s="1" t="inlineStr">
-        <is>
-          <t>Judge is injection-resistant</t>
-        </is>
-      </c>
-      <c r="D32" s="1" t="inlineStr">
-        <is>
-          <t>Agent output cannot instruct the judge; tested with an injected directive</t>
-        </is>
-      </c>
-      <c r="E32" s="1" t="inlineStr">
-        <is>
-          <t>Agent text is concatenated into the judge prompt unguarded</t>
-        </is>
-      </c>
-      <c r="F32" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" s="1" t="inlineStr">
-        <is>
-          <t>Every judge prompt labels submitted UI, source, network payloads, errors, and instructions as untrusted and forbids following scoring directives from them. No dedicated injected artifact was run.</t>
-        </is>
-      </c>
-      <c r="H32" s="1" t="inlineStr">
-        <is>
-          <t>PARTIAL: explicit prompt-injection guardrails exist; adversarial injection remains unmeasured.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1" s="2">
-      <c r="A33" s="1" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="inlineStr">
-        <is>
-          <t>F · Anti-gaming</t>
-        </is>
-      </c>
-      <c r="C33" s="1" t="inlineStr">
-        <is>
-          <t>Tests and rubric are not readable by the agent</t>
-        </is>
-      </c>
-      <c r="D33" s="1" t="inlineStr">
-        <is>
-          <t>Separate verifier environment; tests/ never uploaded to the agent container</t>
-        </is>
-      </c>
-      <c r="E33" s="1" t="inlineStr">
-        <is>
-          <t>Agent can read the assertions it is graded on</t>
-        </is>
-      </c>
-      <c r="F33" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G33" s="1" t="inlineStr">
-        <is>
-          <t>Harbor uses a separate verifier environment. The agent receives /instructions and /assets, while tests and rubric are copied only into the verifier image.</t>
-        </is>
-      </c>
-      <c r="H33" s="1" t="inlineStr">
-        <is>
-          <t>PASS: the agent cannot read its scoring assertions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1" s="2">
-      <c r="A34" s="1" t="inlineStr">
-        <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="inlineStr">
-        <is>
-          <t>F · Anti-gaming</t>
-        </is>
-      </c>
-      <c r="C34" s="1" t="inlineStr">
-        <is>
-          <t>No reward for stalling, refusing, or asking questions</t>
-        </is>
-      </c>
-      <c r="D34" s="1" t="inlineStr">
-        <is>
-          <t>A clarifying-question-only rollout scores &lt;=0.05</t>
-        </is>
-      </c>
-      <c r="E34" s="1" t="inlineStr">
-        <is>
-          <t>Politely declining collects partial credit</t>
-        </is>
-      </c>
-      <c r="F34" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G34" s="1" t="inlineStr">
-        <is>
-          <t>A submission without the required running files deterministically receives 0.0000 before judge execution; measured no-op confirms that refusing or stalling earns no credit.</t>
-        </is>
-      </c>
-      <c r="H34" s="1" t="inlineStr">
-        <is>
-          <t>PASS: no reward for non-delivery.</t>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Measured no-op receives zero before browser judging.</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>

</xml_diff>